<commit_message>
Updated MEX_grids_kan model - 2026-04-22 21:35
</commit_message>
<xml_diff>
--- a/VerveStacks_MEX_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_MEX_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_MEX_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F1D2F31-CD6B-4E46-BD9A-1A6BDC502AF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5AAC6ED3-1F15-4E44-9B40-98A702496A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5299,7 +5299,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07815FAA-8544-4710-8DB5-6B5593F95C48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D57F46AE-1BB7-4871-A035-C2C7FC4FAFD0}">
   <dimension ref="B9:H371"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -32923,7 +32923,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E65DCBF-7181-4513-A563-C3B10B6D8F60}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE1B7F61-C6EB-485A-B1DB-1CB786EE777B}">
   <dimension ref="B9:L371"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated MEX_grids_kan model - 2026-04-22 22:09
</commit_message>
<xml_diff>
--- a/VerveStacks_MEX_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_MEX_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_MEX_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5AAC6ED3-1F15-4E44-9B40-98A702496A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{305279E7-61A7-458D-9CB2-CB92E5177AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5299,7 +5299,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D57F46AE-1BB7-4871-A035-C2C7FC4FAFD0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C80F4AD1-E4AC-48AE-9584-EB16EE6DB1D7}">
   <dimension ref="B9:H371"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -32923,7 +32923,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE1B7F61-C6EB-485A-B1DB-1CB786EE777B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B3475AE-9F69-4D80-8C40-2DA7A2A339E1}">
   <dimension ref="B9:L371"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>